<commit_message>
Enhance AR3.ino and main_cnc.py with improved control logic and UI features
</commit_message>
<xml_diff>
--- a/Laporan_Milling_CNC.xlsx
+++ b/Laporan_Milling_CNC.xlsx
@@ -138,7 +138,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7315200" cy="6410325"/>
+    <ext cx="6686550" cy="6172200"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -466,7 +466,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10 May 2026, 17:12:15</t>
+          <t>19 June 2026, 21:54:46</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10 May 2026, 17:12:32</t>
+          <t>19 June 2026, 21:54:57</t>
         </is>
       </c>
     </row>

</xml_diff>